<commit_message>
Los datos de Wyscout al 28/09/2026
18 de 20 equipos con el layout ALL (109 columnas) y los jugadores del lote 3 (Castilla, Murcia, Zaragoza, Sant Andreu, Teruel, Villarreal B y Rayo/Jaén). Real Madrid Castilla y Real Murcia, y los lotes 1 y 2 de jugadores, se quedan con la descarga completa del 25/09: hoy Wyscout colgaba la pestaña en esos equipos y los lotes nuevos salían sin cuatro equipos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/data/wys/Team Stats Cartagena.xlsx
+++ b/public/data/wys/Team Stats Cartagena.xlsx
@@ -2083,7 +2083,7 @@
         <v>1</v>
       </c>
       <c r="H6" s="0" t="n">
-        <v>0.44</v>
+        <v>0.43</v>
       </c>
       <c r="I6" s="0" t="n">
         <v>9.0</v>
@@ -2095,25 +2095,25 @@
         <v>22.22</v>
       </c>
       <c r="L6" s="0" t="n">
-        <v>315.0</v>
+        <v>314.0</v>
       </c>
       <c r="M6" s="0" t="n">
-        <v>233.0</v>
+        <v>235.0</v>
       </c>
       <c r="N6" s="0" t="n">
-        <v>73.97</v>
+        <v>74.84</v>
       </c>
       <c r="O6" s="0" t="n">
-        <v>37.08</v>
+        <v>37.14</v>
       </c>
       <c r="P6" s="0" t="n">
-        <v>126.0</v>
+        <v>123.0</v>
       </c>
       <c r="Q6" s="0" t="n">
         <v>35.0</v>
       </c>
       <c r="R6" s="0" t="n">
-        <v>46.0</v>
+        <v>43.0</v>
       </c>
       <c r="S6" s="0" t="n">
         <v>45.0</v>
@@ -2131,13 +2131,13 @@
         <v>10.0</v>
       </c>
       <c r="X6" s="0" t="n">
-        <v>129.0</v>
+        <v>150.0</v>
       </c>
       <c r="Y6" s="0" t="n">
-        <v>67.0</v>
+        <v>74.0</v>
       </c>
       <c r="Z6" s="0" t="n">
-        <v>51.94</v>
+        <v>49.33</v>
       </c>
       <c r="AA6" s="0" t="n">
         <v>4.0</v>
@@ -2212,31 +2212,31 @@
         <v>29.41</v>
       </c>
       <c r="AY6" s="0" t="n">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
       <c r="AZ6" s="0" t="n">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
       <c r="BA6" s="0" t="n">
-        <v>17.0</v>
+        <v>18.0</v>
       </c>
       <c r="BB6" s="0" t="n">
         <v>4.0</v>
       </c>
       <c r="BC6" s="0" t="n">
-        <v>7.0</v>
+        <v>8.0</v>
       </c>
       <c r="BD6" s="0" t="n">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
       <c r="BE6" s="0" t="n">
-        <v>48.0</v>
+        <v>53.0</v>
       </c>
       <c r="BF6" s="0" t="n">
-        <v>19.0</v>
+        <v>18.0</v>
       </c>
       <c r="BG6" s="0" t="n">
-        <v>39.58</v>
+        <v>33.96</v>
       </c>
       <c r="BH6" s="0" t="n">
         <v>0.0</v>
@@ -2254,22 +2254,22 @@
         <v>31.25</v>
       </c>
       <c r="BM6" s="0" t="n">
-        <v>46.0</v>
+        <v>55.0</v>
       </c>
       <c r="BN6" s="0" t="n">
-        <v>26.0</v>
+        <v>30.0</v>
       </c>
       <c r="BO6" s="0" t="n">
-        <v>56.52</v>
+        <v>54.55</v>
       </c>
       <c r="BP6" s="0" t="n">
-        <v>21.0</v>
+        <v>24.0</v>
       </c>
       <c r="BQ6" s="0" t="n">
-        <v>12.0</v>
+        <v>15.0</v>
       </c>
       <c r="BR6" s="0" t="n">
-        <v>57.14</v>
+        <v>62.5</v>
       </c>
       <c r="BS6" s="0" t="n">
         <v>0.0</v>
@@ -2281,7 +2281,7 @@
         <v>0</v>
       </c>
       <c r="BV6" s="0" t="n">
-        <v>57.0</v>
+        <v>56.0</v>
       </c>
       <c r="BW6" s="0" t="n">
         <v>36.0</v>
@@ -2299,37 +2299,37 @@
         <v>121.0</v>
       </c>
       <c r="CB6" s="0" t="n">
-        <v>73.0</v>
+        <v>75.0</v>
       </c>
       <c r="CC6" s="0" t="n">
-        <v>60.33</v>
+        <v>61.98</v>
       </c>
       <c r="CD6" s="0" t="n">
-        <v>42.0</v>
+        <v>41.0</v>
       </c>
       <c r="CE6" s="0" t="n">
-        <v>36.0</v>
+        <v>35.0</v>
       </c>
       <c r="CF6" s="0" t="n">
-        <v>85.71</v>
+        <v>85.37</v>
       </c>
       <c r="CG6" s="0" t="n">
         <v>112.0</v>
       </c>
       <c r="CH6" s="0" t="n">
-        <v>96.0</v>
+        <v>97.0</v>
       </c>
       <c r="CI6" s="0" t="n">
-        <v>85.71</v>
+        <v>86.61</v>
       </c>
       <c r="CJ6" s="0" t="n">
-        <v>57.0</v>
+        <v>56.0</v>
       </c>
       <c r="CK6" s="0" t="n">
-        <v>26.0</v>
+        <v>27.0</v>
       </c>
       <c r="CL6" s="0" t="n">
-        <v>45.61</v>
+        <v>48.21</v>
       </c>
       <c r="CM6" s="0" t="n">
         <v>44.0</v>
@@ -2341,13 +2341,13 @@
         <v>50.0</v>
       </c>
       <c r="CP6" s="0" t="n">
-        <v>49.0</v>
+        <v>51.0</v>
       </c>
       <c r="CQ6" s="0" t="n">
-        <v>31.0</v>
+        <v>34.0</v>
       </c>
       <c r="CR6" s="0" t="n">
-        <v>63.27</v>
+        <v>66.67</v>
       </c>
       <c r="CS6" s="0" t="n">
         <v>0.0</v>
@@ -2371,19 +2371,19 @@
         <v>8.0</v>
       </c>
       <c r="CZ6" s="0" t="n">
-        <v>17.07</v>
+        <v>16.96</v>
       </c>
       <c r="DA6" s="0" t="n">
-        <v>3.12</v>
+        <v>3.11</v>
       </c>
       <c r="DB6" s="0" t="n">
-        <v>18.1</v>
+        <v>17.83</v>
       </c>
       <c r="DC6" s="0" t="n">
         <v>19.13</v>
       </c>
       <c r="DD6" s="0" t="n">
-        <v>22.11</v>
+        <v>22.05</v>
       </c>
       <c r="DE6" s="0" t="n">
         <v>18.89</v>
@@ -2443,7 +2443,7 @@
         <v>85.01</v>
       </c>
       <c r="O7" s="0" t="n">
-        <v>62.92</v>
+        <v>62.86</v>
       </c>
       <c r="P7" s="0" t="n">
         <v>129.0</v>
@@ -2458,25 +2458,25 @@
         <v>67.0</v>
       </c>
       <c r="T7" s="0" t="n">
-        <v>77.0</v>
+        <v>78.0</v>
       </c>
       <c r="U7" s="0" t="n">
         <v>29.0</v>
       </c>
       <c r="V7" s="0" t="n">
-        <v>31.0</v>
+        <v>32.0</v>
       </c>
       <c r="W7" s="0" t="n">
         <v>17.0</v>
       </c>
       <c r="X7" s="0" t="n">
-        <v>129.0</v>
+        <v>150.0</v>
       </c>
       <c r="Y7" s="0" t="n">
-        <v>59.0</v>
+        <v>73.0</v>
       </c>
       <c r="Z7" s="0" t="n">
-        <v>45.74</v>
+        <v>48.67</v>
       </c>
       <c r="AA7" s="0" t="n">
         <v>8.0</v>
@@ -2569,13 +2569,13 @@
         <v>23.0</v>
       </c>
       <c r="BE7" s="0" t="n">
-        <v>46.0</v>
+        <v>55.0</v>
       </c>
       <c r="BF7" s="0" t="n">
-        <v>20.0</v>
+        <v>25.0</v>
       </c>
       <c r="BG7" s="0" t="n">
-        <v>43.48</v>
+        <v>45.45</v>
       </c>
       <c r="BH7" s="0" t="n">
         <v>1.0</v>
@@ -2593,22 +2593,22 @@
         <v>22.22</v>
       </c>
       <c r="BM7" s="0" t="n">
-        <v>48.0</v>
+        <v>53.0</v>
       </c>
       <c r="BN7" s="0" t="n">
-        <v>29.0</v>
+        <v>35.0</v>
       </c>
       <c r="BO7" s="0" t="n">
-        <v>60.42</v>
+        <v>66.04</v>
       </c>
       <c r="BP7" s="0" t="n">
-        <v>21.0</v>
+        <v>24.0</v>
       </c>
       <c r="BQ7" s="0" t="n">
         <v>9.0</v>
       </c>
       <c r="BR7" s="0" t="n">
-        <v>42.86</v>
+        <v>37.5</v>
       </c>
       <c r="BS7" s="0" t="n">
         <v>1.0</v>
@@ -2710,7 +2710,7 @@
         <v>7.0</v>
       </c>
       <c r="CZ7" s="0" t="n">
-        <v>16.83</v>
+        <v>16.81</v>
       </c>
       <c r="DA7" s="0" t="n">
         <v>5.27</v>

</xml_diff>